<commit_message>
Fix generic filler descriptions in Unit 13 coding questions
Same fix as prior units, completing the pass across Units 2-13:
rewrote the 10 placeholder descriptions with a real scenario and
explicit logic, verified against existing solutions/test cases.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Question Bank/Coding Questions/Unit 13 - Debugging/Unit 13 - Debugging - Coding Questions.xlsx
+++ b/content/Question Bank/Coding Questions/Unit 13 - Debugging/Unit 13 - Debugging - Coding Questions.xlsx
@@ -1900,7 +1900,8 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Inclusive Loop Fix. Read the input values and print the required result exactly.
+          <t>A ticket-numbering script should print every ticket number from 1 to N, one per line, but a common off-by-one bug is writing the loop as `range(1, n)`, which stops one short and misses ticket N entirely. Write the correct version.
+Write a program that reads a whole number N and prints every whole number from 1 to N, inclusive, one per line, using `range(1, n + 1)`. If N is 0 or less, print nothing.
 ### Input Format
 - Line 1: N
 ### Output Format
@@ -1909,9 +1910,11 @@
 2
 3
 ```
+### Example Walkthrough
+In the sample, N is 3. The correct range `range(1, 4)` produces 1, 2, and 3, so the program prints all three, including the final ticket number 3 that the buggy `range(1, 3)` would have missed.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1998,7 +2001,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr">
         <is>
           <t>5</t>
@@ -2074,16 +2076,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Average Formula Fix. Read the input values and print the required result exactly.
+          <t>A grading script computes the class average from a list of scores, but a common bug is dividing the sum by the wrong count, such as a hardcoded number of students, instead of the actual number of scores that were entered. Write the correct version.
+Write a program that reads a line of space-separated numbers and prints their average, computed as the sum of the numbers divided by exactly how many numbers were entered.
 ### Input Format
-- Line 1: Integers
+- Line 1: Space-separated numbers
 ### Output Format
 ```
 2.0
 ```
+### Example Walkthrough
+In the sample, the numbers are `1 2 3`. Their sum is 6 and there are 3 of them, so the average is 6 / 3 = 2.0, which the program prints.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3674,16 +3679,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Assert Positive. Read the input values and print the required result exactly.
+          <t>A configuration loader uses an assertion to guarantee that a setting value is a positive number before continuing, catching the resulting `AssertionError` to report a friendly message instead of letting the program crash with a raw traceback.
+Write a program that reads a whole number inside a `try` block, uses `assert n &gt; 0` to check it is positive, and prints `OK` if the assertion passes. If the assertion fails, catch the `AssertionError` and print `Not positive`.
 ### Input Format
-- Line 1: Number
+- Line 1: A whole number
 ### Output Format
 ```
 OK
 ```
+### Example Walkthrough
+In the sample, the number is 1, which is positive, so the assertion passes and the program prints `OK`. A value of `0` or lower would fail the assertion and print `Not positive` instead.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3829,16 +3837,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Boundary Pass Fix. Read the input values and print the required result exactly.
+          <t>A results checker marks students as passing at exactly 40 marks or above, but a common bug is using `&gt;` instead of `&gt;=`, which would incorrectly fail a student who scored exactly 40. Write the correct version.
+Write a program that reads a whole number of marks and prints `Pass` if the marks are 40 or more (using `&gt;=`, so exactly 40 counts as a pass), and `Fail` otherwise.
 ### Input Format
 - Line 1: Marks
 ### Output Format
 ```
 Pass
 ```
+### Example Walkthrough
+In the sample, the marks are exactly 40. Using `&gt;=`, 40 is greater than or equal to 40, so the program prints `Pass`, unlike a buggy `&gt;` check which would have incorrectly printed `Fail`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5274,16 +5285,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Sorted Assertion. Read the input values and print the required result exactly.
+          <t>A leaderboard update script assumes an incoming list of scores is already sorted before merging it with the existing leaderboard, and uses an assertion to immediately catch the moment that assumption is violated instead of silently producing a broken leaderboard.
+Write a program that reads a line of space-separated whole numbers inside a `try` block, uses `assert nums == sorted(nums)` to check the list is sorted from smallest to largest, and prints `Sorted` if the assertion passes. If it fails, catch the `AssertionError` and print `Not sorted`.
 ### Input Format
-- Line 1: Integers
+- Line 1: Space-separated whole numbers
 ### Output Format
 ```
 Sorted
 ```
+### Example Walkthrough
+In the sample, the numbers are `1 2 3`, which are already in increasing order, so the assertion passes and the program prints `Sorted`. Numbers like `3 2 1` would fail the assertion and print `Not sorted` instead.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -5429,16 +5443,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for First Zero Trace. Read the input values and print the required result exactly.
+          <t>A sensor log analyzer needs to find the position of the first zero reading in a batch, since a zero often indicates the sensor briefly disconnected, so an engineer traces through the values to find the index of the first occurrence, or -1 if none of the readings were zero.
+Write a program that reads a line of space-separated whole numbers and prints the index (starting at 0) of the first value equal to 0. If no value is 0, print `-1`.
 ### Input Format
-- Line 1: Integers
+- Line 1: Space-separated whole numbers
 ### Output Format
 ```
 1
 ```
+### Example Walkthrough
+In the sample, the readings are `1 0 2`. The first 0 appears at index 1 (the second position, counting from 0), so the program prints `1`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -5585,17 +5602,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Logging Level Count. Read the input values and print the required result exactly.
+          <t>A log-monitoring dashboard scans a batch of log entries and counts exactly how many are tagged with the level `ERROR` (matching the exact case used by the logging system, so `error` in lower case does not count), so it can flag a spike in errors.
+Write a program that reads a whole number N, then reads N more lines each containing a log level, and prints how many of them are exactly `ERROR`.
 ### Input Format
-- Line 1: N
-- Next N lines: Log level
+- Line 1: N, the number of log entries
+- Next N lines: a log level each
 ### Output Format
 ```
 2
 ```
+### Example Walkthrough
+In the sample, N is 3 with the levels `INFO`, `ERROR`, and `ERROR`. Two of the three entries are exactly `ERROR`, so the program prints `2`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- N is a valid whole number matching the number of lines that follow.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7089,17 +7109,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Off By One Window. Read the input values and print the required result exactly.
+          <t>A stock-analysis tool finds the best K-day rolling sum of daily profits to spot the strongest short streak, sliding a window of size K across the data. A common off-by-one bug stops the sliding window one position too early and misses the very last possible window; write the correct version.
+Write a program that reads a line of space-separated whole numbers, reads a whole number K on the next line, and prints the maximum sum of any K consecutive numbers in the list, making sure to check every possible window including the last one.
 ### Input Format
-- Line 1: Integers
-- Line 2: K
+- Line 1: Space-separated whole numbers
+- Line 2: K, the window size
 ### Output Format
 ```
 7
 ```
+### Example Walkthrough
+In the sample, the numbers are `1 2 3 4` and K is 2. The possible windows of size 2 are `1+2=3`, `2+3=5`, and `3+4=7`; the largest is 7, so the program prints `7`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- K is a valid whole number no greater than the number of values given.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -7252,16 +7275,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Invariant Stack. Read the input values and print the required result exactly.
+          <t>A browser's back-button history is modeled as a stack of push and pop operations coming from user navigation actions. The invariant that must always hold is that you can't pop when the stack is empty (you can't go back further than the history allows), so the app validates a sequence of operations to check whether it ever breaks that rule.
+Write a program that reads a line of space-separated operations (`push` or `pop`), simulates them on a stack, and prints `OK` if every `pop` had something to remove, or `Broken` the moment a `pop` is attempted on an empty stack.
 ### Input Format
-- Line 1: Operations
+- Line 1: Space-separated operations (`push` or `pop`)
 ### Output Format
 ```
 OK
 ```
+### Example Walkthrough
+In the sample, the operations are `push pop`. The `push` adds an item, and the `pop` removes it since the stack wasn't empty, so the invariant holds and the program prints `OK`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- The input is a valid line of space-separated operations, each either `push` or `pop`.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -7411,18 +7437,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A supplemental Python practice task for Rubber Duck Trace. Read the input values and print the required result exactly.
+          <t>While rubber-duck debugging a budgeting script, a developer traces through it line by line: for each new expense added, print the running total so far immediately, to see exactly where the total starts to go wrong.
+Write a program that reads a line of space-separated whole numbers and, keeping a running total, prints the total after adding each number, one line per number.
 ### Input Format
-- Line 1: Integers
+- Line 1: Space-separated whole numbers
 ### Output Format
 ```
 1
 3
 6
 ```
+### Example Walkthrough
+In the sample, the numbers are `1 2 3`. After adding 1, the running total is 1; after adding 2, it becomes 3; after adding 3, it becomes 6 - so the program prints `1`, then `3`, then `6`.
 ### Constraints
-- Inputs follow the described format.
-- Print exactly the requested output with no extra text.</t>
+- All numeric inputs are valid whole numbers in the ranges implied by the examples.
+- Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>